<commit_message>
Rename Falkland Is. to Falkland Islands (Malvinas), log in CHANGES
</commit_message>
<xml_diff>
--- a/terrestrial/CHANGES_20-Aug-26.xlsx
+++ b/terrestrial/CHANGES_20-Aug-26.xlsx
@@ -176,7 +176,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -240,6 +240,9 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -519,7 +522,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F53"/>
+  <dimension ref="A1:F55"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="14.453125" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="9.08984375" customWidth="1" style="19" min="1" max="1"/>
@@ -1269,8 +1272,32 @@
         </is>
       </c>
     </row>
-    <row r="54" ht="15.75" customHeight="1" s="19"/>
-    <row r="55" ht="15.75" customHeight="1" s="19"/>
+    <row r="54" ht="15.75" customHeight="1" s="19">
+      <c r="A54" s="10" t="n">
+        <v>9</v>
+      </c>
+      <c r="B54" s="7" t="inlineStr">
+        <is>
+          <t>ANTARCTIC</t>
+        </is>
+      </c>
+      <c r="D54" s="4" t="n"/>
+    </row>
+    <row r="55" ht="15.75" customHeight="1" s="19">
+      <c r="A55" s="26" t="n">
+        <v>90</v>
+      </c>
+      <c r="B55" s="4" t="inlineStr">
+        <is>
+          <t>Subantarctic Islands</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>N Falkland Islands (Malvinas) (Falkland Is.) FAL</t>
+        </is>
+      </c>
+    </row>
     <row r="56" ht="15.75" customHeight="1" s="19"/>
     <row r="57" ht="15.75" customHeight="1" s="19"/>
     <row r="58" ht="15.75" customHeight="1" s="19"/>

</xml_diff>